<commit_message>
feat: harder water treatment domain, difficulty field, recalibrated presets
Rebuild the water treatment domain from an easy linear DAG into a
genuinely hard causal discovery problem: time-series with feedback loop,
latent confounder (Source_Water_Quality), nonlinear edges (saturating,
quadratic, piecewise, interaction), Simpson's paradox, MNAR sensor
censoring, regime change, and lagged rainfall effect. Pilot study now
has partial compliance instead of perfectly fixed dose.

Add optional `difficulty` field (easy|medium|hard|expert) to
ExperimentConfig and set it in all domain YAMLs. The TUI launcher now
reads difficulty dynamically from experiment.yaml instead of a hardcoded
dictionary.

Recalibrate preset and max_iterations per domain:
- toy_function: fast/3, alien_minerals: default/5, alloy_design: default/5
- water_treatment: high/8, spo2: max/10

Reclassify spo2 from Hard to Expert in README.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/domains/water_treatment/seed/data/data_dictionary.xlsx
+++ b/domains/water_treatment/seed/data/data_dictionary.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -488,12 +488,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CHEM_D_MGL</t>
+          <t>ORG_LOAD_MGL</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Chemical Dose</t>
+          <t>Organic Load</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -505,85 +505,102 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>FLOW_M3H</t>
+          <t>CHEM_D_MGL</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Flow Rate</t>
+          <t>Chemical Dose</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>m³/h</t>
+          <t>mg/L</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>RES_T_MIN</t>
+          <t>FLOW_M3H</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Residence Time</t>
+          <t>Flow Rate</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>min</t>
+          <t>m³/h</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>FLOC_UM</t>
+          <t>RES_T_MIN</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Floc Size</t>
+          <t>Residence Time</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>µm</t>
+          <t>min</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SETL_MH</t>
+          <t>FLOC_UM</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Settling Rate</t>
+          <t>Floc Size</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>m/h</t>
+          <t>µm</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>OUT_CLR_NTU</t>
+          <t>SETL_MH</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>Settling Rate</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>m/h</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>OUT_CLR</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>Outlet Clarity</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>NTU</t>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>index</t>
         </is>
       </c>
     </row>
@@ -598,7 +615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -649,6 +666,30 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Source water</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Upstream construction project began ~mid-2024. Possible impact on intake water.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Operators adjust chemical dosing based on incoming water conditions and recent output quality.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>